<commit_message>
commiting the project backup
</commit_message>
<xml_diff>
--- a/server/data/canteen_data.xlsx
+++ b/server/data/canteen_data.xlsx
@@ -400,7 +400,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F10"/>
+  <dimension ref="A1:F12"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -436,7 +436,7 @@
         <v>25</v>
       </c>
       <c r="E2" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="3">
@@ -504,7 +504,10 @@
         <v>70</v>
       </c>
       <c r="E6" t="b">
-        <v>1</v>
+        <v>0</v>
+      </c>
+      <c r="F6" t="str">
+        <v>COMSES AT 4 AGAIN</v>
       </c>
     </row>
     <row r="7">
@@ -575,16 +578,50 @@
         <v>1</v>
       </c>
     </row>
+    <row r="11">
+      <c r="A11" t="str">
+        <v>ITM010</v>
+      </c>
+      <c r="B11" t="str">
+        <v>VEG BIRYANI</v>
+      </c>
+      <c r="C11" t="str">
+        <v>FASTFOOD</v>
+      </c>
+      <c r="D11">
+        <v>200</v>
+      </c>
+      <c r="E11" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="str">
+        <v>ITM011</v>
+      </c>
+      <c r="B12" t="str">
+        <v>MASALA DOSA WITH KARAM</v>
+      </c>
+      <c r="C12" t="str">
+        <v>South Indian</v>
+      </c>
+      <c r="D12">
+        <v>49</v>
+      </c>
+      <c r="E12" t="b">
+        <v>1</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:F10"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:F12"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:H14"/>
+  <dimension ref="A1:H22"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -950,16 +987,224 @@
         <v>2026-08-21T06:48:18.287Z</v>
       </c>
     </row>
+    <row r="15">
+      <c r="A15" t="str">
+        <v>1001</v>
+      </c>
+      <c r="B15" t="str">
+        <v>2026-08-24</v>
+      </c>
+      <c r="C15" t="str">
+        <v>[{"item_id":"ITM001","name":"Veg Puff","price":25,"qty":4}]</v>
+      </c>
+      <c r="D15">
+        <v>100</v>
+      </c>
+      <c r="E15" t="str">
+        <v>pay_test_1787561120533_qhoxf</v>
+      </c>
+      <c r="F15" t="str">
+        <v>PAID</v>
+      </c>
+      <c r="G15" t="str">
+        <v>SERVED</v>
+      </c>
+      <c r="H15" t="str">
+        <v>2026-08-24T08:45:20.547Z</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="str">
+        <v>1002</v>
+      </c>
+      <c r="B16" t="str">
+        <v>2026-08-24</v>
+      </c>
+      <c r="C16" t="str">
+        <v>[{"item_id":"ITM002","name":"Samosa (2 pcs)","price":30,"qty":1}]</v>
+      </c>
+      <c r="D16">
+        <v>30</v>
+      </c>
+      <c r="E16" t="str">
+        <v>pay_test_1787561228806_hj40f</v>
+      </c>
+      <c r="F16" t="str">
+        <v>PAID</v>
+      </c>
+      <c r="G16" t="str">
+        <v>SERVED</v>
+      </c>
+      <c r="H16" t="str">
+        <v>2026-08-24T08:47:08.834Z</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="str">
+        <v>1003</v>
+      </c>
+      <c r="B17" t="str">
+        <v>2026-08-24</v>
+      </c>
+      <c r="C17" t="str">
+        <v>[{"item_id":"ITM002","name":"Samosa (2 pcs)","price":30,"qty":1}]</v>
+      </c>
+      <c r="D17">
+        <v>30</v>
+      </c>
+      <c r="E17" t="str">
+        <v>sim_pay_1787561540534_0_n9p8</v>
+      </c>
+      <c r="F17" t="str">
+        <v>PAID</v>
+      </c>
+      <c r="G17" t="str">
+        <v>PLACED</v>
+      </c>
+      <c r="H17" t="str">
+        <v>2026-08-24T08:52:20.545Z</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="str">
+        <v>1004</v>
+      </c>
+      <c r="B18" t="str">
+        <v>2026-08-24</v>
+      </c>
+      <c r="C18" t="str">
+        <v>[{"item_id":"ITM002","name":"Samosa (2 pcs)","price":30,"qty":1}]</v>
+      </c>
+      <c r="D18">
+        <v>30</v>
+      </c>
+      <c r="E18" t="str">
+        <v>sim_pay_1787561540534_1_q9lm</v>
+      </c>
+      <c r="F18" t="str">
+        <v>PAID</v>
+      </c>
+      <c r="G18" t="str">
+        <v>PLACED</v>
+      </c>
+      <c r="H18" t="str">
+        <v>2026-08-24T08:52:20.615Z</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="str">
+        <v>1005</v>
+      </c>
+      <c r="B19" t="str">
+        <v>2026-08-24</v>
+      </c>
+      <c r="C19" t="str">
+        <v>[{"item_id":"ITM002","name":"Samosa (2 pcs)","price":30,"qty":1}]</v>
+      </c>
+      <c r="D19">
+        <v>30</v>
+      </c>
+      <c r="E19" t="str">
+        <v>sim_pay_1787561540534_2_ino3</v>
+      </c>
+      <c r="F19" t="str">
+        <v>PAID</v>
+      </c>
+      <c r="G19" t="str">
+        <v>PLACED</v>
+      </c>
+      <c r="H19" t="str">
+        <v>2026-08-24T08:52:20.666Z</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="str">
+        <v>1006</v>
+      </c>
+      <c r="B20" t="str">
+        <v>2026-08-24</v>
+      </c>
+      <c r="C20" t="str">
+        <v>[{"item_id":"ITM002","name":"Samosa (2 pcs)","price":30,"qty":1}]</v>
+      </c>
+      <c r="D20">
+        <v>30</v>
+      </c>
+      <c r="E20" t="str">
+        <v>sim_pay_1787561540534_3_lhbk</v>
+      </c>
+      <c r="F20" t="str">
+        <v>PAID</v>
+      </c>
+      <c r="G20" t="str">
+        <v>PLACED</v>
+      </c>
+      <c r="H20" t="str">
+        <v>2026-08-24T08:52:20.726Z</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="str">
+        <v>1007</v>
+      </c>
+      <c r="B21" t="str">
+        <v>2026-08-24</v>
+      </c>
+      <c r="C21" t="str">
+        <v>[{"item_id":"ITM002","name":"Samosa (2 pcs)","price":30,"qty":1}]</v>
+      </c>
+      <c r="D21">
+        <v>30</v>
+      </c>
+      <c r="E21" t="str">
+        <v>sim_pay_1787561540534_4_vzpx</v>
+      </c>
+      <c r="F21" t="str">
+        <v>PAID</v>
+      </c>
+      <c r="G21" t="str">
+        <v>PLACED</v>
+      </c>
+      <c r="H21" t="str">
+        <v>2026-08-24T08:52:20.781Z</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="str">
+        <v>1008</v>
+      </c>
+      <c r="B22" t="str">
+        <v>2026-08-24</v>
+      </c>
+      <c r="C22" t="str">
+        <v>[{"item_id":"ITM001","name":"Veg Puff","price":25,"qty":1}]</v>
+      </c>
+      <c r="D22">
+        <v>25</v>
+      </c>
+      <c r="E22" t="str">
+        <v>sim_pay_1787561580919_0_2mfo</v>
+      </c>
+      <c r="F22" t="str">
+        <v>PAID</v>
+      </c>
+      <c r="G22" t="str">
+        <v>PLACED</v>
+      </c>
+      <c r="H22" t="str">
+        <v>2026-08-24T08:53:00.959Z</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:H14"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:H22"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:B2"/>
+  <dimension ref="A1:B3"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -977,9 +1222,17 @@
         <v>29</v>
       </c>
     </row>
+    <row r="3">
+      <c r="A3" t="str">
+        <v>2026-08-24</v>
+      </c>
+      <c r="B3">
+        <v>8</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:B2"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:B3"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -1005,6 +1258,7 @@
       </c>
     </row>
   </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <ignoredErrors>
     <ignoredError numberStoredAsText="1" sqref="A1:B2"/>
   </ignoredErrors>

</xml_diff>